<commit_message>
Student import: B.Tech only - skip M.Tech rows, four-year batches
The portal covers two B.Tech batches (2023-27 and 2024-28). A JNTU No with
"1D" (M.Tech) is now an Error row in both the full student import and the
results update, with the single reason "M.Tech students are not
imported." (no department/section noise). Batches are always four years,
so no 2024-26 batch is ever created, and the VLSI&ES department/aliases
are gone from DepartmentAliasSeeder. Fixture and tests updated.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/tests/Fixtures/college_students_synthetic.xlsx
+++ b/backend/tests/Fixtures/college_students_synthetic.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="84">
   <si>
     <t>Name</t>
   </si>
@@ -244,9 +244,6 @@
   </si>
   <si>
     <t>24341D5702</t>
-  </si>
-  <si>
-    <t>VLSI &amp; ES</t>
   </si>
   <si>
     <t>Ravi Test</t>
@@ -1216,7 +1213,7 @@
         <v>18</v>
       </c>
       <c r="E5" t="s">
-        <v>76</v>
+        <v>14</v>
       </c>
       <c r="F5" t="s">
         <v>19</v>
@@ -1239,19 +1236,19 @@
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B6" t="s">
         <v>77</v>
-      </c>
-      <c r="B6" t="s">
-        <v>78</v>
       </c>
       <c r="D6" t="s">
         <v>23</v>
       </c>
       <c r="E6" t="s">
+        <v>78</v>
+      </c>
+      <c r="F6" t="s">
         <v>79</v>
-      </c>
-      <c r="F6" t="s">
-        <v>80</v>
       </c>
       <c r="G6">
         <v>9876500017</v>
@@ -1271,10 +1268,10 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
+        <v>80</v>
+      </c>
+      <c r="B7" t="s">
         <v>81</v>
-      </c>
-      <c r="B7" t="s">
-        <v>82</v>
       </c>
       <c r="C7">
         <v>2023</v>
@@ -1283,10 +1280,10 @@
         <v>29</v>
       </c>
       <c r="E7" t="s">
+        <v>82</v>
+      </c>
+      <c r="F7" t="s">
         <v>83</v>
-      </c>
-      <c r="F7" t="s">
-        <v>84</v>
       </c>
       <c r="H7">
         <v>8.6</v>

</xml_diff>